<commit_message>
docs: skala flowchart pas dengan kolom Pelaksana di Word dan Excel
</commit_message>
<xml_diff>
--- a/docs/SOP_PENGGUNAAN_ARUMANIS.xlsx
+++ b/docs/SOP_PENGGUNAAN_ARUMANIS.xlsx
@@ -3038,15 +3038,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1130300</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>550545</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3063,8 +3063,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="2844800" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="4457700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3081,15 +3081,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3106,8 +3106,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3124,15 +3124,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3149,8 +3149,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3167,15 +3167,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3192,8 +3192,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3210,15 +3210,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3235,8 +3235,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3253,15 +3253,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3278,8 +3278,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3296,15 +3296,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3321,8 +3321,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3339,15 +3339,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3364,8 +3364,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3382,15 +3382,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3407,8 +3407,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3425,15 +3425,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3450,8 +3450,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3468,15 +3468,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3493,8 +3493,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3511,15 +3511,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3536,8 +3536,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1800225"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1743075"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3554,15 +3554,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3579,8 +3579,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3597,15 +3597,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3622,8 +3622,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3640,15 +3640,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3665,8 +3665,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3683,15 +3683,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3708,8 +3708,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3726,15 +3726,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3751,8 +3751,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3769,15 +3769,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3794,8 +3794,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3812,15 +3812,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3837,8 +3837,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3855,15 +3855,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3880,8 +3880,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3898,15 +3898,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3923,8 +3923,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3941,15 +3941,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3966,8 +3966,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3984,15 +3984,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4009,8 +4009,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1800225"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1743075"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4027,15 +4027,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4052,8 +4052,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4070,15 +4070,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4095,8 +4095,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4113,15 +4113,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4138,8 +4138,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4156,15 +4156,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4181,8 +4181,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4199,15 +4199,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4224,8 +4224,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4242,15 +4242,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4267,8 +4267,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4285,15 +4285,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4310,8 +4310,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4328,15 +4328,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4353,8 +4353,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4371,15 +4371,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4396,8 +4396,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4414,15 +4414,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4439,8 +4439,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4457,15 +4457,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4482,8 +4482,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1800225"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1743075"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4500,15 +4500,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4525,8 +4525,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4543,15 +4543,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4568,8 +4568,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4586,15 +4586,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4611,8 +4611,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4629,15 +4629,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4654,8 +4654,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4672,15 +4672,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4697,8 +4697,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4715,15 +4715,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4740,8 +4740,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4758,15 +4758,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4783,8 +4783,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4801,15 +4801,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4826,8 +4826,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4844,15 +4844,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>518160</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>169545</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4869,8 +4869,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="3413760" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="3714750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4887,15 +4887,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4912,8 +4912,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4930,15 +4930,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4955,8 +4955,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4973,15 +4973,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4998,8 +4998,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5016,15 +5016,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5041,8 +5041,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5059,15 +5059,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5084,8 +5084,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5102,15 +5102,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5127,8 +5127,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5145,15 +5145,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5170,8 +5170,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5188,15 +5188,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5213,8 +5213,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5231,15 +5231,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5256,8 +5256,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5274,15 +5274,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5299,8 +5299,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5317,15 +5317,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5342,8 +5342,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5360,15 +5360,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5385,8 +5385,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5403,15 +5403,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5428,8 +5428,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1800225"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1743075"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5446,15 +5446,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1130300</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>550545</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5471,8 +5471,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="2844800" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="4457700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5489,15 +5489,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5514,8 +5514,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5532,15 +5532,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5557,8 +5557,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5575,15 +5575,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5600,8 +5600,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5618,15 +5618,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5643,8 +5643,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5661,15 +5661,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>113919</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5686,8 +5686,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4389120" cy="3209544"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2228850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5704,15 +5704,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5729,8 +5729,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5747,15 +5747,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5772,8 +5772,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5790,15 +5790,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5815,8 +5815,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1990725"/>
-          <a:ext cx="4267200" cy="4160520"/>
+          <a:off x="2628900" y="1933575"/>
+          <a:ext cx="1790700" cy="2971800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7474,7 +7474,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -7496,7 +7496,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -7518,7 +7518,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -7540,7 +7540,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -7761,7 +7761,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -7783,7 +7783,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -7960,7 +7960,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -8004,7 +8004,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -8203,7 +8203,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -8247,7 +8247,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -8269,7 +8269,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -8446,7 +8446,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -8468,7 +8468,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -8490,7 +8490,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -8512,7 +8512,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -8689,7 +8689,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -8733,7 +8733,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -8932,7 +8932,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -8954,7 +8954,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -9153,7 +9153,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -9197,7 +9197,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -9398,7 +9398,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -9420,7 +9420,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -9444,7 +9444,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -9643,7 +9643,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -9665,7 +9665,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -9687,7 +9687,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -9711,7 +9711,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -9733,7 +9733,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -10388,7 +10388,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -10410,7 +10410,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -10432,7 +10432,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -10456,7 +10456,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -10677,7 +10677,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -10723,7 +10723,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -10745,7 +10745,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -10944,7 +10944,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -10966,7 +10966,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -10990,7 +10990,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -11012,7 +11012,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -11189,7 +11189,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -11233,7 +11233,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -11257,7 +11257,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -11279,7 +11279,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -11456,7 +11456,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -11478,7 +11478,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -11500,7 +11500,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -11524,7 +11524,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -11546,7 +11546,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -11745,7 +11745,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -11767,7 +11767,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -11944,7 +11944,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -11966,7 +11966,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -11988,7 +11988,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -12012,7 +12012,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -12034,7 +12034,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -12211,7 +12211,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -12233,7 +12233,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -12255,7 +12255,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -12279,7 +12279,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -12301,7 +12301,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -12478,7 +12478,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -12522,7 +12522,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -12546,7 +12546,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -12568,7 +12568,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -12745,7 +12745,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -12767,7 +12767,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -12789,7 +12789,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -12811,7 +12811,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -12988,7 +12988,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -13010,7 +13010,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -13032,7 +13032,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -13056,7 +13056,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -13078,7 +13078,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -13100,7 +13100,7 @@
       </c>
       <c r="J12" s="12"/>
     </row>
-    <row r="13" spans="1:10" ht="58" customHeight="1">
+    <row r="13" spans="1:10" ht="58.5" customHeight="1">
       <c r="A13" s="11" t="s">
         <v>341</v>
       </c>
@@ -13277,7 +13277,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -13299,7 +13299,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -13321,7 +13321,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -13498,7 +13498,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -13542,7 +13542,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -13719,7 +13719,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -13741,7 +13741,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -13763,7 +13763,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -13787,7 +13787,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -13809,7 +13809,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -13986,7 +13986,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -14008,7 +14008,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -14030,7 +14030,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -14054,7 +14054,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -14076,7 +14076,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -14253,7 +14253,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -14275,7 +14275,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -14297,7 +14297,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -14321,7 +14321,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -14343,7 +14343,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -14520,7 +14520,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -14542,7 +14542,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -14564,7 +14564,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -14763,7 +14763,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -14785,7 +14785,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -14807,7 +14807,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -14829,7 +14829,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -15006,7 +15006,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -15028,7 +15028,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -15050,7 +15050,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -15072,7 +15072,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -15249,7 +15249,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -15271,7 +15271,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -15293,7 +15293,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -15315,7 +15315,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -15492,7 +15492,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -15514,7 +15514,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -15536,7 +15536,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -15558,7 +15558,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -15721,7 +15721,7 @@
       </c>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="58" customHeight="1">
+    <row r="7" spans="1:10" ht="58.5" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>319</v>
       </c>
@@ -15743,7 +15743,7 @@
       </c>
       <c r="J7" s="12"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>323</v>
       </c>
@@ -15765,7 +15765,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>328</v>
       </c>
@@ -15787,7 +15787,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>334</v>
       </c>
@@ -15809,7 +15809,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>338</v>
       </c>
@@ -15987,7 +15987,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -16009,7 +16009,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -16031,7 +16031,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -16055,7 +16055,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -16077,7 +16077,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -16254,7 +16254,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -16276,7 +16276,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -16298,7 +16298,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -16475,7 +16475,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -16497,7 +16497,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -16519,7 +16519,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -16543,7 +16543,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -16565,7 +16565,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -16742,7 +16742,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -16764,7 +16764,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -16786,7 +16786,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -16810,7 +16810,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -16832,7 +16832,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -17009,7 +17009,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -17031,7 +17031,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -17053,7 +17053,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -17077,7 +17077,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -17099,7 +17099,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -17276,7 +17276,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -17298,7 +17298,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -17320,7 +17320,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -17344,7 +17344,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -17366,7 +17366,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -17543,7 +17543,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -17565,7 +17565,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -17587,7 +17587,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -17611,7 +17611,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -17633,7 +17633,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -17810,7 +17810,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -17832,7 +17832,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -17854,7 +17854,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -17878,7 +17878,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -17900,7 +17900,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -18099,7 +18099,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -18121,7 +18121,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -18143,7 +18143,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -18320,7 +18320,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -18342,7 +18342,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -18364,7 +18364,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -18386,7 +18386,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -18549,7 +18549,7 @@
       </c>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="58" customHeight="1">
+    <row r="7" spans="1:10" ht="58.5" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>319</v>
       </c>
@@ -18571,7 +18571,7 @@
       </c>
       <c r="J7" s="12"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>323</v>
       </c>
@@ -18593,7 +18593,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>328</v>
       </c>
@@ -18615,7 +18615,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>334</v>
       </c>
@@ -18791,7 +18791,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -18813,7 +18813,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -18835,7 +18835,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -18859,7 +18859,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -18881,7 +18881,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -19058,7 +19058,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -19080,7 +19080,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -19102,7 +19102,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -19279,7 +19279,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -19301,7 +19301,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -19323,7 +19323,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -19500,7 +19500,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -19522,7 +19522,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -19544,7 +19544,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -19566,7 +19566,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -19743,7 +19743,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -19765,7 +19765,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -19787,7 +19787,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -19964,7 +19964,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -19986,7 +19986,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -20008,7 +20008,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -20030,7 +20030,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -20207,7 +20207,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -20229,7 +20229,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -20251,7 +20251,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -20273,7 +20273,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -20450,7 +20450,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -20472,7 +20472,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -20494,7 +20494,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -20671,7 +20671,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -20693,7 +20693,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -20715,7 +20715,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -20737,7 +20737,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -20914,7 +20914,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -20936,7 +20936,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -20958,7 +20958,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -20980,7 +20980,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -21143,7 +21143,7 @@
       </c>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="58" customHeight="1">
+    <row r="7" spans="1:10" ht="58.5" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>319</v>
       </c>
@@ -21165,7 +21165,7 @@
       </c>
       <c r="J7" s="12"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>323</v>
       </c>
@@ -21187,7 +21187,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>328</v>
       </c>
@@ -21209,7 +21209,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>334</v>
       </c>
@@ -21231,7 +21231,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>338</v>
       </c>
@@ -21407,7 +21407,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -21429,7 +21429,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -21451,7 +21451,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -21628,7 +21628,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -21650,7 +21650,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -21672,7 +21672,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -21849,7 +21849,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -21871,7 +21871,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -21893,7 +21893,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -21915,7 +21915,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -21937,7 +21937,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="58" customHeight="1">
+    <row r="12" spans="1:10" ht="58.5" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>338</v>
       </c>
@@ -21959,7 +21959,7 @@
       </c>
       <c r="J12" s="12"/>
     </row>
-    <row r="13" spans="1:10" ht="58" customHeight="1">
+    <row r="13" spans="1:10" ht="58.5" customHeight="1">
       <c r="A13" s="11" t="s">
         <v>341</v>
       </c>
@@ -22136,7 +22136,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -22158,7 +22158,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -22180,7 +22180,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -22202,7 +22202,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -22379,7 +22379,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -22401,7 +22401,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -22423,7 +22423,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -22445,7 +22445,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -22622,7 +22622,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -22644,7 +22644,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -22666,7 +22666,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -22843,7 +22843,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -22865,7 +22865,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -22887,7 +22887,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -23064,7 +23064,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -23108,7 +23108,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -23285,7 +23285,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -23307,7 +23307,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -23329,7 +23329,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -23353,7 +23353,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>
@@ -23516,7 +23516,7 @@
       </c>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="58" customHeight="1">
+    <row r="7" spans="1:10" ht="58.5" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>319</v>
       </c>
@@ -23538,7 +23538,7 @@
       </c>
       <c r="J7" s="12"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>323</v>
       </c>
@@ -23560,7 +23560,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>328</v>
       </c>
@@ -23736,7 +23736,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="58" customHeight="1">
+    <row r="8" spans="1:10" ht="58.5" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>319</v>
       </c>
@@ -23758,7 +23758,7 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="58" customHeight="1">
+    <row r="9" spans="1:10" ht="58.5" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>323</v>
       </c>
@@ -23780,7 +23780,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="58" customHeight="1">
+    <row r="10" spans="1:10" ht="58.5" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>328</v>
       </c>
@@ -23802,7 +23802,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="58" customHeight="1">
+    <row r="11" spans="1:10" ht="58.5" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>334</v>
       </c>

</xml_diff>